<commit_message>
docs(fix-style): sprint 7 couleur
</commit_message>
<xml_diff>
--- a/docs/pilotage/equipe-09-sprint-backlog-v5.0.xlsx
+++ b/docs/pilotage/equipe-09-sprint-backlog-v5.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="14"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="10"/>
   </bookViews>
   <sheets>
     <sheet name="Garde" sheetId="1" state="visible" r:id="rId3"/>
@@ -1264,7 +1264,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1346,13 +1346,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFD7D7"/>
-        <bgColor rgb="FFDEE6EF"/>
+        <bgColor rgb="FFF7D1D5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF5CE"/>
         <bgColor rgb="FFFFFFD7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7D1D5"/>
+        <bgColor rgb="FFFFD7D7"/>
       </patternFill>
     </fill>
   </fills>
@@ -1420,7 +1426,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1645,6 +1651,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1701,13 +1711,13 @@
       <rgbColor rgb="FFDDE8CB"/>
       <rgbColor rgb="FFFFE994"/>
       <rgbColor rgb="FFDEE6EF"/>
-      <rgbColor rgb="FFFFFBEB"/>
+      <rgbColor rgb="FFFFD7D7"/>
       <rgbColor rgb="FFF8FAFC"/>
-      <rgbColor rgb="FFFFD7D7"/>
+      <rgbColor rgb="FFF7D1D5"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFFFBEB"/>
       <rgbColor rgb="FFF59E0B"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF475569"/>
@@ -3615,94 +3625,94 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="40.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="55" t="s">
+      <c r="A24" s="56" t="s">
         <v>288</v>
       </c>
-      <c r="B24" s="55" t="s">
+      <c r="B24" s="56" t="s">
         <v>297</v>
       </c>
-      <c r="C24" s="55" t="s">
+      <c r="C24" s="56" t="s">
         <v>298</v>
       </c>
-      <c r="D24" s="55" t="s">
+      <c r="D24" s="56" t="s">
         <v>141</v>
       </c>
-      <c r="E24" s="55" t="n">
+      <c r="E24" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="F24" s="55" t="n">
+      <c r="F24" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="G24" s="55" t="s">
+      <c r="G24" s="56" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="41.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="55" t="s">
+      <c r="A25" s="56" t="s">
         <v>288</v>
       </c>
-      <c r="B25" s="55" t="s">
+      <c r="B25" s="56" t="s">
         <v>299</v>
       </c>
-      <c r="C25" s="55" t="s">
+      <c r="C25" s="56" t="s">
         <v>300</v>
       </c>
-      <c r="D25" s="55" t="s">
+      <c r="D25" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="E25" s="55" t="n">
+      <c r="E25" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="F25" s="55" t="n">
+      <c r="F25" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="55" t="s">
+      <c r="G25" s="56" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="55" t="s">
+      <c r="A26" s="56" t="s">
         <v>288</v>
       </c>
-      <c r="B26" s="55" t="s">
+      <c r="B26" s="56" t="s">
         <v>301</v>
       </c>
-      <c r="C26" s="55" t="s">
+      <c r="C26" s="56" t="s">
         <v>302</v>
       </c>
-      <c r="D26" s="55" t="s">
+      <c r="D26" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="E26" s="55" t="n">
+      <c r="E26" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="F26" s="55" t="n">
+      <c r="F26" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="55" t="s">
+      <c r="G26" s="56" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="55" t="s">
+      <c r="A27" s="56" t="s">
         <v>288</v>
       </c>
-      <c r="B27" s="55" t="s">
+      <c r="B27" s="56" t="s">
         <v>303</v>
       </c>
-      <c r="C27" s="55" t="s">
+      <c r="C27" s="56" t="s">
         <v>304</v>
       </c>
-      <c r="D27" s="55" t="s">
+      <c r="D27" s="56" t="s">
         <v>73</v>
       </c>
-      <c r="E27" s="55" t="n">
+      <c r="E27" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="F27" s="55" t="n">
+      <c r="F27" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="G27" s="55" t="s">
+      <c r="G27" s="56" t="s">
         <v>268</v>
       </c>
     </row>
@@ -3989,104 +3999,104 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="56" t="s">
+      <c r="B6" s="57" t="s">
         <v>311</v>
       </c>
-      <c r="C6" s="57" t="s">
+      <c r="C6" s="58" t="s">
         <v>312</v>
       </c>
-      <c r="D6" s="56" t="s">
+      <c r="D6" s="57" t="s">
         <v>313</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="56" t="s">
+      <c r="B7" s="57" t="s">
         <v>314</v>
       </c>
-      <c r="C7" s="57" t="s">
+      <c r="C7" s="58" t="s">
         <v>312</v>
       </c>
-      <c r="D7" s="56" t="s">
+      <c r="D7" s="57" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="56" t="s">
+      <c r="B8" s="57" t="s">
         <v>316</v>
       </c>
-      <c r="C8" s="57" t="s">
+      <c r="C8" s="58" t="s">
         <v>312</v>
       </c>
-      <c r="D8" s="56" t="s">
+      <c r="D8" s="57" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="56" t="s">
+      <c r="B9" s="57" t="s">
         <v>318</v>
       </c>
-      <c r="C9" s="57" t="s">
+      <c r="C9" s="58" t="s">
         <v>312</v>
       </c>
-      <c r="D9" s="56" t="s">
+      <c r="D9" s="57" t="s">
         <v>319</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="56" t="s">
+      <c r="B10" s="57" t="s">
         <v>320</v>
       </c>
-      <c r="C10" s="57" t="s">
+      <c r="C10" s="58" t="s">
         <v>312</v>
       </c>
-      <c r="D10" s="56"/>
+      <c r="D10" s="57"/>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="56" t="s">
+      <c r="B11" s="57" t="s">
         <v>321</v>
       </c>
-      <c r="C11" s="57" t="s">
+      <c r="C11" s="58" t="s">
         <v>312</v>
       </c>
-      <c r="D11" s="56" t="s">
+      <c r="D11" s="57" t="s">
         <v>322</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="56" t="s">
+      <c r="B12" s="57" t="s">
         <v>323</v>
       </c>
-      <c r="C12" s="57" t="s">
+      <c r="C12" s="58" t="s">
         <v>312</v>
       </c>
-      <c r="D12" s="56"/>
+      <c r="D12" s="57"/>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="56" t="s">
+      <c r="B13" s="57" t="s">
         <v>324</v>
       </c>
-      <c r="C13" s="57" t="s">
+      <c r="C13" s="58" t="s">
         <v>312</v>
       </c>
-      <c r="D13" s="56"/>
+      <c r="D13" s="57"/>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="56" t="s">
+      <c r="B14" s="57" t="s">
         <v>325</v>
       </c>
-      <c r="C14" s="57" t="s">
+      <c r="C14" s="58" t="s">
         <v>312</v>
       </c>
-      <c r="D14" s="56"/>
+      <c r="D14" s="57"/>
     </row>
     <row r="15" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="56" t="s">
+      <c r="B15" s="57" t="s">
         <v>326</v>
       </c>
-      <c r="C15" s="57" t="s">
+      <c r="C15" s="58" t="s">
         <v>312</v>
       </c>
-      <c r="D15" s="56" t="s">
+      <c r="D15" s="57" t="s">
         <v>327</v>
       </c>
     </row>

</xml_diff>